<commit_message>
Epic har fået tilføjet status Tester for CC version 5.0 og ACK 2.0. EDI Portalen har fået tilføjet Godkendt for CC version 5.0
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F3F4245-8040-4801-839D-F54EBB54E980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6D1A70-F3C3-45A2-A28C-F93D2A28EE54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 02-02-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 20-02-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 02-02-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 20-02-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Planner4You har fået status Godkendt
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6D1A70-F3C3-45A2-A28C-F93D2A28EE54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB6C632D-2135-4A7F-B786-EAC7449BC4B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 20-02-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 04-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 20-02-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 04-03-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Vena har fået status Godkendt for ACK og CC
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB6C632D-2135-4A7F-B786-EAC7449BC4B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC1244DF-3052-46B2-8DCB-F5863AFE125B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 04-03-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 06-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 04-03-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 06-03-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
MADS har fået status Tester for VANSEnvelope
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5CFAA09-0B09-4A0D-88D8-6FA4CF5F2786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB078AA-1F27-4449-8DF4-D53DECCB2850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14625" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 06-03-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 09-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 06-03-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 09-03-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
SYNLAB har fået status Tester for CC, ACK og VANSEnvelope
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB078AA-1F27-4449-8DF4-D53DECCB2850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F080342-25F8-492C-BA62-3FEA5ECBDDA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14625" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 09-03-2026" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Vena har fået status Tester for APD-DK
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F080342-25F8-492C-BA62-3FEA5ECBDDA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A623D14-2088-41B5-B405-BDC839EA35C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 09-03-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 11-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 09-03-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 11-03-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Confirma har fået overtaget TM Care's registreringer.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F705335-856B-4190-B704-8A9C484E21C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7947D0A-C1F7-47B6-BDEB-DB8EE2BE7714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 11-03-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 20-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 11-03-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 20-03-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
sundhed.dk har fået tilføjet status Tester for afsendelse af DIS91 og modtagelse af CTL01-03.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7947D0A-C1F7-47B6-BDEB-DB8EE2BE7714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73277A93-48A5-41F0-8AEA-671C61C84606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 20-03-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 25-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 20-03-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 25-03-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
XMedicus har som LPS fået markeringer.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73277A93-48A5-41F0-8AEA-671C61C84606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC77E66E-3237-48B6-B3FD-0D7D8E43E533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 25-03-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 08-04-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 25-03-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 08-04-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Netforvaltning sundhed har fået status Godkendt for standarder.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC77E66E-3237-48B6-B3FD-0D7D8E43E533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{233D62BF-D3B6-4F60-9245-0B804AD04CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 08-04-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 10-04-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 08-04-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 10-04-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Opdateret med status og ny testleder på forløb.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D87EA20-9853-42E5-B1D2-7E77BD6D4368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A387FA-141F-4ABD-9ABC-E12D6620390D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15045" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 10-04-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 14-04-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 10-04-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 14-04-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
ViTolker har fået tilføjet status tester for RUC37 og CTL01-03
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A387FA-141F-4ABD-9ABC-E12D6620390D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82823EDA-70CB-47A9-99EB-889C4ECE2FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 14-04-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 24-04-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 14-04-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 24-04-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Nexta har fået status godkendt for RUC03
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBF1CBF7-3E50-4199-BF72-23795A2BF910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3997EF31-D4B3-4E32-AC8A-9F951C5F30DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 27-04-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 06-05-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 27-04-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 06-05-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Sundhed.dk har fået status Tester for modtagelse af SER (2.0) og XDS Metadata (1.0)
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3997EF31-D4B3-4E32-AC8A-9F951C5F30DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BFBFE07-FEBD-4FAC-B804-96068E530EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 06-05-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 01-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 06-05-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 01-06-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Novax og sdk har fået status Tester for ECN og XDS Metadata.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089002D6-14B6-4C54-A3A7-F5A3AD880BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A14CAF1-24CF-4AF2-B08E-E068F9EB6FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 02-06-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 05-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 02-06-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 05-06-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
HejDoktor og BCC godkendt
HejDoktor og BCC godkendt
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hua\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B222D356-985D-4AEB-82D2-AFCFAB377DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9162A97C-3B24-4596-B622-3E5F4D6864E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3150" yWindow="3135" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 29-01-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 09-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 29-01-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 09-06-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
ViTolker har fået status Godkendt for RUC37 og CTL01-03
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hua\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{767C80DB-C682-4214-8EFA-0CA5D597E977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3BE33D-9479-457C-8A25-8FCD9CDB784E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 09-06-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 15-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 09-06-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 15-06-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
XMedicus har fået status godkendt for modtagelse af RPT01 som LPS.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3BE33D-9479-457C-8A25-8FCD9CDB784E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DF510E-A0C5-4B47-B59E-58FE0059E332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 15-06-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 22-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 15-06-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 22-06-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
MUSE for Nord, Midt og Syd har fået status tester for Shared EKG og XDS Metadata.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DF510E-A0C5-4B47-B59E-58FE0059E332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C10F9C-6BA3-49BE-B93F-657717E09A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 22-06-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 23-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 22-06-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 23-06-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Clinio Medical har fået status Tester for standarder.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C10F9C-6BA3-49BE-B93F-657717E09A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E681A7-580E-4EBF-BEE0-CF83EC16442D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 23-06-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 25-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 23-06-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 25-06-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Systematic Cura har fået status Godkendt for CC og ACK
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E25979-9728-4E7A-A27C-4334887F5D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301C791D-3084-48D6-A60A-67A885B6DC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 30-06-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 01-07-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 30-06-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 01-07-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Columna CIS har fået status Godkendt for CC og ACK
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301C791D-3084-48D6-A60A-67A885B6DC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3B03F7-FF81-4EF6-9D5E-A8948C4A0EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 01-07-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 03-07-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 01-07-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 03-07-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
HejDoktor har fået tilføjet status Tester for henvisningsstandarder.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EBF2831-7BD6-4172-BE2A-B30F44DE37E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B7566B-E9C5-4344-8E1F-0FAC16BD80E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="945" windowWidth="21600" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 19-08-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 21-08-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 19-08-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 21-08-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Vena har fået status Tester ifm. GGOP afsendelse.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B7566B-E9C5-4344-8E1F-0FAC16BD80E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295E320D-3E56-4AC2-8025-7383194E824C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4560" yWindow="945" windowWidth="21600" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 21-08-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 27-08-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 21-08-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 27-08-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -422,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -458,7 +458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -475,7 +475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -489,7 +489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -506,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -523,7 +523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -540,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -557,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
DokuDok har fået status Tester for Batch 1
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295E320D-3E56-4AC2-8025-7383194E824C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467F9BB8-DA14-4BF4-9514-989D5F8AEC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 27-08-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 02-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 27-08-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 02-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Vena har fået status Tester for RUC10, DIS10 og REF10
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467F9BB8-DA14-4BF4-9514-989D5F8AEC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CBDE6A4-BCC4-4D75-98C6-4A6B8941798B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14625" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 02-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 06-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 02-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 06-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Vena har fået status Tester for DIS90
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A6051F-67D5-4761-A14D-69673ED1B14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B67999-4C33-4669-8176-6D78BBFF38E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14625" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 06-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 07-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 06-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 07-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>

<commit_message>
Vena [SPL] har fået status godkendt for speciallæge-standarder.
</commit_message>
<xml_diff>
--- a/html/Apotekssystemer_excel.XLSX
+++ b/html/Apotekssystemer_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B67999-4C33-4669-8176-6D78BBFF38E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5970323-5C0D-47C3-940B-8807E362540D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 07-09-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 09-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Apotekssystemer">'Opdateret d. 07-09-2026'!$A$1:$E$9</definedName>
+    <definedName name="Apotekssystemer">'Opdateret d. 09-09-2026'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>

</xml_diff>